<commit_message>
feat(brand): adopt Concept C logo, add favicons, webmanifest, and purge legacy ReviewBoost references
</commit_message>
<xml_diff>
--- a/restaurants_whatsapp_leads.xlsx
+++ b/restaurants_whatsapp_leads.xlsx
@@ -398,21 +398,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M51"/>
-  <cols>
-    <col min="1" max="1" width="6.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
-    <col min="5" max="5" width="25.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="35.83203125" customWidth="1"/>
-    <col min="8" max="8" width="38.83203125" customWidth="1"/>
-    <col min="9" max="9" width="45.83203125" customWidth="1"/>
-    <col min="10" max="10" width="30.83203125" customWidth="1"/>
-    <col min="11" max="11" width="45.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="65.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -504,7 +489,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -556,7 +541,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
@@ -608,7 +593,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="5" xml:space="preserve">
@@ -660,7 +645,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="6" xml:space="preserve">
@@ -712,7 +697,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
@@ -764,7 +749,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="8" xml:space="preserve">
@@ -816,7 +801,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="9" xml:space="preserve">
@@ -868,7 +853,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="10" xml:space="preserve">
@@ -920,7 +905,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="11" xml:space="preserve">
@@ -972,7 +957,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="12" xml:space="preserve">
@@ -1024,7 +1009,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="13" xml:space="preserve">
@@ -1076,7 +1061,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="14" xml:space="preserve">
@@ -1128,7 +1113,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="15" xml:space="preserve">
@@ -1180,7 +1165,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="16" xml:space="preserve">
@@ -1232,7 +1217,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="17" xml:space="preserve">
@@ -1284,7 +1269,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="18" xml:space="preserve">
@@ -1336,7 +1321,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="19" xml:space="preserve">
@@ -1388,7 +1373,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="20" xml:space="preserve">
@@ -1440,7 +1425,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="21" xml:space="preserve">
@@ -1492,7 +1477,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="22" xml:space="preserve">
@@ -1544,7 +1529,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="23" xml:space="preserve">
@@ -1596,7 +1581,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="24" xml:space="preserve">
@@ -1648,7 +1633,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="25" xml:space="preserve">
@@ -1700,7 +1685,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="26" xml:space="preserve">
@@ -1752,7 +1737,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="27" xml:space="preserve">
@@ -1804,7 +1789,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="28" xml:space="preserve">
@@ -1856,7 +1841,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="29" xml:space="preserve">
@@ -1908,7 +1893,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="30" xml:space="preserve">
@@ -1960,7 +1945,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="31" xml:space="preserve">
@@ -2012,7 +1997,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="32" xml:space="preserve">
@@ -2064,7 +2049,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="33" xml:space="preserve">
@@ -2116,7 +2101,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="34" xml:space="preserve">
@@ -2168,7 +2153,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="35" xml:space="preserve">
@@ -2220,7 +2205,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="36" xml:space="preserve">
@@ -2272,7 +2257,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="37" xml:space="preserve">
@@ -2324,7 +2309,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="38" xml:space="preserve">
@@ -2376,7 +2361,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="39" xml:space="preserve">
@@ -2428,7 +2413,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="40" xml:space="preserve">
@@ -2480,7 +2465,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="41" xml:space="preserve">
@@ -2532,7 +2517,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="42" xml:space="preserve">
@@ -2584,7 +2569,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="43" xml:space="preserve">
@@ -2636,7 +2621,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="44" xml:space="preserve">
@@ -2688,7 +2673,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="45" xml:space="preserve">
@@ -2740,7 +2725,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="46" xml:space="preserve">
@@ -2792,7 +2777,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="47" xml:space="preserve">
@@ -2844,7 +2829,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="48" xml:space="preserve">
@@ -2896,7 +2881,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="49" xml:space="preserve">
@@ -2948,7 +2933,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="50" xml:space="preserve">
@@ -3000,7 +2985,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
     <row r="51" xml:space="preserve">
@@ -3052,7 +3037,7 @@
 Can I send a printed 4x6" acrylic table standee over to your manager to test this week?
 Best regards,
 Anurag Mishra
-Sayalabs &amp; ReviewBoost (scanner.sayalabs.in)</v>
+Sayalabs &amp; Credo (scanner.sayalabs.in)</v>
       </c>
     </row>
   </sheetData>

</xml_diff>